<commit_message>
data: publish 2026-10-17 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-17-182路.xlsx
+++ b/data/export/2026-10-17-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC10"/>
+  <dimension ref="A1:AC17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,7 +441,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -632,32 +632,36 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:13</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>68分钟</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr"/>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -665,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -689,33 +693,37 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>1/11</t>
         </is>
       </c>
     </row>
@@ -743,32 +751,36 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>70分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -776,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -800,33 +812,37 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA3" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>70.0</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>2/11</t>
         </is>
       </c>
     </row>
@@ -854,32 +870,36 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>74分钟</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -887,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -911,33 +931,37 @@
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA4" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>74.0</t>
+        </is>
+      </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>4/11</t>
         </is>
       </c>
     </row>
@@ -965,32 +989,36 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:47</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>72分钟</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -998,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1022,33 +1050,37 @@
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA5" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>3/11</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1141,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1148,7 +1180,7 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr">
@@ -1159,7 +1191,7 @@
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/11</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1252,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1270,7 +1302,7 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/11</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1363,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1381,7 +1413,7 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/11</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1474,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1492,7 +1524,7 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/11</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1585,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1603,7 +1635,800 @@
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:42</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>—/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>1/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A66513D</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>70.0</t>
+        </is>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>2/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A67983D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>74.0</t>
+        </is>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>4/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A32298D</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>—/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>—/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>08:10</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>08:10</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>3/11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-10-17 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-17-182路.xlsx
+++ b/data/export/2026-10-17-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC48"/>
+  <dimension ref="A1:AC50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>5/11</t>
+          <t>6/11</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1498,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="Z9" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA9" s="2" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1661,17 +1661,17 @@
       </c>
       <c r="AA10" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
-          <t>75.7</t>
+          <t>74.2</t>
         </is>
       </c>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>7/11</t>
+          <t>5/11</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="AC11" s="2" t="inlineStr">
         <is>
-          <t>6/11</t>
+          <t>7/11</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AA12" s="2" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
-          <t>77.2</t>
+          <t>77.5</t>
         </is>
       </c>
       <c r="AC15" s="2" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="AC18" s="2" t="inlineStr">
         <is>
-          <t>5/11</t>
+          <t>6/11</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="Z20" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA20" s="2" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="AC21" s="2" t="inlineStr">
         <is>
-          <t>6/11</t>
+          <t>7/11</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -3085,17 +3085,17 @@
       </c>
       <c r="AA22" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
-          <t>75.7</t>
+          <t>74.2</t>
         </is>
       </c>
       <c r="AC22" s="2" t="inlineStr">
         <is>
-          <t>7/11</t>
+          <t>5/11</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3160,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3328,7 +3328,7 @@
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
-          <t>77.2</t>
+          <t>77.5</t>
         </is>
       </c>
       <c r="AC24" s="2" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -3874,7 +3874,7 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -3928,7 +3928,7 @@
       </c>
       <c r="AC29" s="2" t="inlineStr">
         <is>
-          <t>5/11</t>
+          <t>6/11</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
@@ -4037,17 +4037,17 @@
       </c>
       <c r="AA30" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
-          <t>75.7</t>
+          <t>74.2</t>
         </is>
       </c>
       <c r="AC30" s="2" t="inlineStr">
         <is>
-          <t>7/11</t>
+          <t>5/11</t>
         </is>
       </c>
     </row>
@@ -4166,7 +4166,7 @@
       </c>
       <c r="AC31" s="2" t="inlineStr">
         <is>
-          <t>6/11</t>
+          <t>7/11</t>
         </is>
       </c>
     </row>
@@ -4231,7 +4231,7 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
@@ -4399,7 +4399,7 @@
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
-          <t>77.2</t>
+          <t>77.5</t>
         </is>
       </c>
       <c r="AC33" s="2" t="inlineStr">
@@ -4588,7 +4588,7 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="Z35" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA35" s="2" t="inlineStr">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="AC36" s="2" t="inlineStr">
         <is>
-          <t>5/11</t>
+          <t>6/11</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4826,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -4999,7 +4999,7 @@
       </c>
       <c r="AC38" s="2" t="inlineStr">
         <is>
-          <t>6/11</t>
+          <t>7/11</t>
         </is>
       </c>
     </row>
@@ -5064,7 +5064,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
@@ -5156,12 +5156,12 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>13:54</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>79分钟</t>
+          <t>80分钟</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
-          <t>77.2</t>
+          <t>77.5</t>
         </is>
       </c>
       <c r="AC40" s="2" t="inlineStr">
@@ -5265,32 +5265,36 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>70分钟</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
       <c r="K41" s="2" t="inlineStr"/>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M41" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -5298,7 +5302,7 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
@@ -5322,17 +5326,17 @@
       </c>
       <c r="W41" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X41" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y41" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z41" s="2" t="inlineStr">
@@ -5342,17 +5346,17 @@
       </c>
       <c r="AA41" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
-          <t>75.7</t>
+          <t>74.2</t>
         </is>
       </c>
       <c r="AC41" s="2" t="inlineStr">
         <is>
-          <t>7/11</t>
+          <t>5/11</t>
         </is>
       </c>
     </row>
@@ -5413,7 +5417,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
@@ -5452,7 +5456,7 @@
       </c>
       <c r="Z42" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA42" s="2" t="inlineStr">
@@ -5528,7 +5532,7 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P43" s="2" t="inlineStr">
@@ -5567,7 +5571,7 @@
       </c>
       <c r="Z43" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AA43" s="2" t="inlineStr">
@@ -5643,7 +5647,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -5758,7 +5762,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -5873,7 +5877,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
@@ -5988,7 +5992,7 @@
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P47" s="2" t="inlineStr">
@@ -6042,7 +6046,7 @@
       </c>
       <c r="AC47" s="2" t="inlineStr">
         <is>
-          <t>5/11</t>
+          <t>6/11</t>
         </is>
       </c>
     </row>
@@ -6103,7 +6107,7 @@
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
@@ -6147,17 +6151,247 @@
       </c>
       <c r="AA48" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
-          <t>75.7</t>
+          <t>74.2</t>
         </is>
       </c>
       <c r="AC48" s="2" t="inlineStr">
         <is>
-          <t>7/11</t>
+          <t>5/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr"/>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>14:52</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr"/>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr"/>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q49" s="2" t="inlineStr"/>
+      <c r="R49" s="2" t="inlineStr"/>
+      <c r="S49" s="2" t="inlineStr"/>
+      <c r="T49" s="2" t="inlineStr"/>
+      <c r="U49" s="2" t="inlineStr">
+        <is>
+          <t>14:52</t>
+        </is>
+      </c>
+      <c r="V49" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W49" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X49" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y49" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z49" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA49" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB49" s="2" t="inlineStr">
+        <is>
+          <t>71.5</t>
+        </is>
+      </c>
+      <c r="AC49" s="2" t="inlineStr">
+        <is>
+          <t>2/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr"/>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr"/>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q50" s="2" t="inlineStr"/>
+      <c r="R50" s="2" t="inlineStr"/>
+      <c r="S50" s="2" t="inlineStr"/>
+      <c r="T50" s="2" t="inlineStr"/>
+      <c r="U50" s="2" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="V50" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W50" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X50" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y50" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z50" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA50" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB50" s="2" t="inlineStr">
+        <is>
+          <t>70.0</t>
+        </is>
+      </c>
+      <c r="AC50" s="2" t="inlineStr">
+        <is>
+          <t>1/11</t>
         </is>
       </c>
     </row>

</xml_diff>